<commit_message>
Listini C75S: ferramenta Maico calcolata per misura dal poolfile WinPlus
- KIT_ANTA: regole FFB/FFH ricavate dall'export MaicoWinPlus del 14/09/2026
  (cremonese, prolunghe, movimenti angolari, chiusure centrali, forbice +
  braccio, asta lato cerniere, cerniera angolare + bandella, scontri fungo)
  con prezzi dal netto 2025; voci fisse modificabili (martellina, nottolino
  personalizzato, semifissa).
- xlsx: foglio FerrGriglia (costo ferramenta per cella) referenziato dalle
  formule; foglio Ferramenta = kit della misura di riferimento.
- HTML: kit mostrato per la misura interrogata, prezzi per codice e voci
  fisse modificabili, griglie e xlsx allineati allo script.
- Verifica: F1 1000x1500 kit 37,34, costo 442,05, listino 1383,62 in
  entrambi; formule xlsx identiche.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YMK4dVsJMS4SCsnwzeiU3b
</commit_message>
<xml_diff>
--- a/listini-c75s/F1_SENZA_VETRO.xlsx
+++ b/listini-c75s/F1_SENZA_VETRO.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Parametri" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Coefficienti" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Ferramenta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="FerrGriglia" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,35 +515,35 @@
         <v>500</v>
       </c>
       <c r="B3" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B2+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C3" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C2+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D3" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D2+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E3" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E2+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F3" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F2+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G3" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G2+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H3" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H2+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I3" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A3)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A3)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A3)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I2+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -551,35 +552,35 @@
         <v>600</v>
       </c>
       <c r="B4" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B3+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C4" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C3+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D4" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D3+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E4" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E3+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F4" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F3+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G4" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G3+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H4" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H3+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I4" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A4)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A4)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A4)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I3+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -588,35 +589,35 @@
         <v>700</v>
       </c>
       <c r="B5" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B4+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C5" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C4+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D5" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D4+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E4+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F5" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F4+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G5" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G4+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H5" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H4+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I5" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A5)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A5)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A5)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I4+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -625,35 +626,35 @@
         <v>800</v>
       </c>
       <c r="B6" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B5+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C6" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C5+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D6" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D5+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E6" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E5+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F6" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F5+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G6" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G5+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H6" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H5+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I6" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A6)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A6)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A6)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I5+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -662,35 +663,35 @@
         <v>900</v>
       </c>
       <c r="B7" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B6+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C7" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C6+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D7" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D6+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E7" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E6+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F7" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F6+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G7" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G6+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H7" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H6+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I7" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A7)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A7)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A7)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I6+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -699,35 +700,35 @@
         <v>1000</v>
       </c>
       <c r="B8" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B7+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C8" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C7+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D8" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D7+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E8" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E7+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F8" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F7+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G8" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G7+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H8" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H7+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I8" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A8)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A8)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A8)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I7+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -736,35 +737,35 @@
         <v>1100</v>
       </c>
       <c r="B9" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B8+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C9" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C8+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D9" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D8+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E9" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E8+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F9" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F8+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G9" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G8+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H9" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H8+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I9" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A9)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A9)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A9)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I8+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -773,35 +774,35 @@
         <v>1200</v>
       </c>
       <c r="B10" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B9+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C10" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C9+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D10" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D9+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E10" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E9+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F10" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F9+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G10" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G9+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H10" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H9+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I10" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A10)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A10)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A10)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I9+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -810,35 +811,35 @@
         <v>1300</v>
       </c>
       <c r="B11" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B10+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C11" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C10+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D11" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D10+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E11" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E10+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F11" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F10+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G11" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G10+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H11" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H10+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I11" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A11)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A11)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A11)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I10+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -847,35 +848,35 @@
         <v>1400</v>
       </c>
       <c r="B12" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C12" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D12" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E12" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F12" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G12" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H12" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I12" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A12)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A12)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A12)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -884,35 +885,35 @@
         <v>1500</v>
       </c>
       <c r="B13" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B12+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C13" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C12+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D13" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D12+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E13" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E12+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F13" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F12+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G13" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G12+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H13" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H12+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I13" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A13)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A13)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A13)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I12+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -921,35 +922,35 @@
         <v>1600</v>
       </c>
       <c r="B14" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B13+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C14" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C13+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D14" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D13+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E14" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E13+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F14" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F13+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G14" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G13+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H14" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H13+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I14" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A14)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A14)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A14)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I13+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -958,35 +959,35 @@
         <v>1700</v>
       </c>
       <c r="B15" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B14+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C15" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C14+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D15" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D14+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E15" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E14+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F15" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F14+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G15" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G14+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H15" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H14+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I15" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A15)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A15)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A15)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I14+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -995,35 +996,35 @@
         <v>1800</v>
       </c>
       <c r="B16" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B15+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C16" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C15+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D16" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D15+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E16" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E15+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F16" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F15+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G16" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G15+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H16" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H15+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I16" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A16)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A16)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A16)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I15+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -1032,35 +1033,35 @@
         <v>1900</v>
       </c>
       <c r="B17" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B16+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C17" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C16+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D17" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D16+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E17" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E16+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F17" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F16+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G17" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G16+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H17" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H16+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I17" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A17)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A17)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A17)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I16+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -1069,35 +1070,35 @@
         <v>2000</v>
       </c>
       <c r="B18" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B17+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="C18" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C17+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="D18" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D17+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="E18" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E17+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="F18" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F17+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="G18" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G17+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="H18" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H17+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
       <c r="I18" s="4">
-        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
+        <f>ROUND(ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$2+Coefficienti!$B$3*$A18)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$2+Coefficienti!$B$6*$A18)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$2+Coefficienti!$B$9*$A18)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I17+Coefficienti!$B$11*Parametri!$B$6,2)*(1+Parametri!$B$7),2)</f>
         <v/>
       </c>
     </row>
@@ -1144,35 +1145,35 @@
         <v>500</v>
       </c>
       <c r="B23" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B2+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C23" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C2+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D23" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D2+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E23" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E2+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F23" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F2+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G23" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G2+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H23" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H2+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I23" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A23)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A23)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A23)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I2+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1181,35 +1182,35 @@
         <v>600</v>
       </c>
       <c r="B24" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B3+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C24" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C3+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D24" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D3+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E24" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E3+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F24" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F3+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G24" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G3+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H24" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H3+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I24" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A24)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A24)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A24)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I3+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1218,35 +1219,35 @@
         <v>700</v>
       </c>
       <c r="B25" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B4+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C25" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C4+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D25" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D4+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E25" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E4+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F25" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F4+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G25" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G4+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H25" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H4+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I25" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A25)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A25)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A25)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I4+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1255,35 +1256,35 @@
         <v>800</v>
       </c>
       <c r="B26" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B5+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C26" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C5+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D26" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D5+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E26" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E5+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F26" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F5+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G26" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G5+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H26" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H5+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I26" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A26)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A26)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A26)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I5+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1292,35 +1293,35 @@
         <v>900</v>
       </c>
       <c r="B27" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B6+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C27" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C6+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D27" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D6+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E27" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E6+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F27" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F6+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G27" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G6+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H27" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H6+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I27" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A27)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A27)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A27)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I6+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1329,35 +1330,35 @@
         <v>1000</v>
       </c>
       <c r="B28" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B7+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C28" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C7+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D28" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D7+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E28" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E7+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F28" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F7+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G28" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G7+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H28" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H7+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I28" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A28)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A28)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A28)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I7+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1366,35 +1367,35 @@
         <v>1100</v>
       </c>
       <c r="B29" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B8+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C29" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C8+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D29" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D8+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E29" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E8+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F29" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F8+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G29" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G8+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H29" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H8+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I29" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A29)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A29)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A29)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I8+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1403,35 +1404,35 @@
         <v>1200</v>
       </c>
       <c r="B30" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B9+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C30" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C9+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D30" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D9+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E30" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E9+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F30" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F9+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G30" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G9+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H30" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H9+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I30" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A30)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A30)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A30)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I9+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1440,35 +1441,35 @@
         <v>1300</v>
       </c>
       <c r="B31" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B10+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C31" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C10+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D31" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D10+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E31" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E10+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F31" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F10+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G31" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G10+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H31" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H10+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I31" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A31)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A31)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A31)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I10+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1477,35 +1478,35 @@
         <v>1400</v>
       </c>
       <c r="B32" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C32" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D32" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E32" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F32" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G32" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H32" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I32" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A32)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A32)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A32)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1514,35 +1515,35 @@
         <v>1500</v>
       </c>
       <c r="B33" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B12+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C33" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C12+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D33" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D12+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E33" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E12+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F33" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F12+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G33" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G12+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H33" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H12+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I33" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A33)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A33)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A33)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I12+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1551,35 +1552,35 @@
         <v>1600</v>
       </c>
       <c r="B34" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B13+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C34" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C13+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D34" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D13+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E34" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E13+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F34" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F13+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G34" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G13+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H34" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H13+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I34" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A34)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A34)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A34)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I13+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1588,35 +1589,35 @@
         <v>1700</v>
       </c>
       <c r="B35" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B14+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C35" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C14+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D35" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D14+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E35" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E14+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F35" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F14+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G35" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G14+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H35" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H14+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I35" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A35)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A35)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A35)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I14+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1625,35 +1626,35 @@
         <v>1800</v>
       </c>
       <c r="B36" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B15+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C36" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C15+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D36" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D15+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E36" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E15+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F36" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F15+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G36" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G15+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H36" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H15+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I36" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A36)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A36)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A36)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I15+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1662,35 +1663,35 @@
         <v>1900</v>
       </c>
       <c r="B37" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B16+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C37" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C16+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D37" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D16+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E37" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E16+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F37" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F16+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G37" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G16+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H37" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H16+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I37" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A37)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A37)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A37)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I16+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -1699,35 +1700,35 @@
         <v>2000</v>
       </c>
       <c r="B38" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*B$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*B$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*B$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!B17+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="C38" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*C$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*C$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*C$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!C17+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="D38" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*D$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*D$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*D$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!D17+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="E38" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*E$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*E$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*E$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!E17+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="F38" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*F$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*F$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*F$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!F17+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="G38" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*G$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*G$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*G$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!G17+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="H38" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*H$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*H$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*H$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!H17+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
       <c r="I38" s="4">
-        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+Ferramenta!$D$11+Coefficienti!$B$11*Parametri!$B$6,2)</f>
+        <f>ROUND((((Coefficienti!$B$1+Coefficienti!$B$2*I$22+Coefficienti!$B$3*$A38)*Parametri!$B$1+(Coefficienti!$B$4+Coefficienti!$B$5*I$22+Coefficienti!$B$6*$A38)*Parametri!$B$2)*(1-Parametri!$B$3)+((Coefficienti!$B$7+Coefficienti!$B$8*I$22+Coefficienti!$B$9*$A38)+Coefficienti!$B$10)*(1-Parametri!$B$4))*(1+Parametri!$B$5)+FerrGriglia!I17+Coefficienti!$B$11*Parametri!$B$6,2)</f>
         <v/>
       </c>
     </row>
@@ -2020,7 +2021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2053,18 +2054,23 @@
           <t>Fonte</t>
         </is>
       </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Kit Maico per la misura di riferimento 1000x1500 (FFB/FFH = anta-20). Le griglie usano il foglio FerrGriglia (kit per ogni misura).</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Martellina DK (1033) — non nel netto 2025</t>
+          <t>Cremonese Multi-Matic (lvMWEspagnoletteGesamt) (201745)</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>5.5</v>
+        <v>3.57</v>
       </c>
       <c r="D2" s="4">
         <f>B2*C2</f>
@@ -2072,21 +2078,21 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>manuale</t>
+          <t>netto 2025</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Cremonese Multi Matic GR1590 (201745)</t>
+          <t>Prolunga cremonese sopra (VerlaengerungFixOben) (201750)</t>
         </is>
       </c>
       <c r="B3" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>3.57</v>
+        <v>2.17</v>
       </c>
       <c r="D3" s="4">
         <f>B3*C3</f>
@@ -2101,14 +2107,14 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Chiusura centrale MM (201752)</t>
+          <t>Prolunga cremonese sotto (VerlaengerungFixUnten) (201750)</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>1.26</v>
+        <v>2.17</v>
       </c>
       <c r="D4" s="4">
         <f>B4*C4</f>
@@ -2123,7 +2129,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Movimento angolare MM (222201)</t>
+          <t>Movimento angolare MM (Eckumlenkung) (222201)</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
@@ -2145,7 +2151,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Movimento angolare prolungabile (222209)</t>
+          <t>Movimento angolare verticale (EckumlenkungVertikal) (222209)</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
@@ -2167,14 +2173,14 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Scontro fungo scost.9 (356361)</t>
+          <t>Chiusura centrale lato cerniere (MittelverschlussEinteiligIS) (211930)</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.3728</v>
+        <v>2.03</v>
       </c>
       <c r="D7" s="4">
         <f>B7*C7</f>
@@ -2189,14 +2195,14 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Scontro nottolino (355866) — NON a listino</t>
+          <t>Chiusura centrale orizzontale (Mittelverschluss) (211929)</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0</v>
+        <v>1.77</v>
       </c>
       <c r="D8" s="4">
         <f>B8*C8</f>
@@ -2204,21 +2210,21 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>da inserire</t>
+          <t>netto 2025</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Cerniere a vista (set anta) — DA INSERIRE</t>
+          <t>Forbice + braccio (ScherenMontiert) (211900)</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>0</v>
+        <v>3.24</v>
       </c>
       <c r="D9" s="4">
         <f>B9*C9</f>
@@ -2226,21 +2232,21 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>da inserire</t>
+          <t>netto 2025</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Forbice a vista + braccio — DA INSERIRE</t>
+          <t>Forbice + braccio (ScherenMontiert) (211901)</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0</v>
+        <v>3.24</v>
       </c>
       <c r="D10" s="4">
         <f>B10*C10</f>
@@ -2248,25 +2254,673 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>da inserire</t>
+          <t>netto 2025</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>TOTALE FERRAMENTA</t>
-        </is>
-      </c>
-      <c r="D11" s="10">
-        <f>SUM(D2:D10)</f>
-        <v/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Asta lato cerniere tagliabile (Drehbandstulp) (202269)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="D11" s="4">
+        <f>B11*C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>netto 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Cerniera angolare (ArtNrEcklager) (250400)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="D12" s="4">
+        <f>B12*C12</f>
+        <v/>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>netto 2025</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>Bandella cerniera angolare (ArtNrEcklagerband) (215806)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D13" s="4">
+        <f>B13*C13</f>
+        <v/>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>netto 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Scontro fungo IS (SchliessteilIS) (356361)</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0.3728</v>
+      </c>
+      <c r="D14" s="4">
+        <f>B14*C14</f>
+        <v/>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>netto 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Martellina DK — non nel netto 2025 (1033)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D15" s="4">
+        <f>B15*C15</f>
+        <v/>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>manuale</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Scontro nottolino personalizzato (VZPersonalisiert) — NON a listino (355866)</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4">
+        <f>B16*C16</f>
+        <v/>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>da inserire</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>TOTALE FERRAMENTA</t>
+        </is>
+      </c>
+      <c r="D17" s="10">
+        <f>SUM(D2:D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
           <t>Celle gialle modificabili. Prezzi a 0 = da inserire: il listino li ignora finché vuoti.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>H/L</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="C1" s="9" t="n">
+        <v>600</v>
+      </c>
+      <c r="D1" s="9" t="n">
+        <v>700</v>
+      </c>
+      <c r="E1" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="F1" s="9" t="n">
+        <v>900</v>
+      </c>
+      <c r="G1" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1" s="9" t="n">
+        <v>1100</v>
+      </c>
+      <c r="I1" s="9" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>22.25</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>25.12</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>28.21</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>28.21</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>29.15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="n">
+        <v>600</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>22.25</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>25.12</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>28.21</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>28.21</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>29.15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="n">
+        <v>700</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>22.25</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>25.12</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>28.21</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>28.21</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>29.15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>22.73</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>25.96</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>25.96</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>28.69</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>28.69</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>29.15</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>29.63</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>900</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>31.67</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>32.03</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>32.03</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>35.22</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>29.52</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>32.39</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>35.94</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>36.42</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>1100</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>29.52</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>32.39</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>32.75</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>35.94</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>36.42</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>30.06</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>32.93</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>33.29</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>33.29</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>36.02</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>36.02</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>36.48</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>36.96</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>1300</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>29.58</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>32.45</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>32.81</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>32.81</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>35.54</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>35.54</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>36.48</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>29.84</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>32.71</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>33.07</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>33.07</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>36.26</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>36.74</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>31.38</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>34.25</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>34.61</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>34.61</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>37.34</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>37.34</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>37.8</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>38.28</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>1600</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>31.53</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>37.49</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>37.49</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>37.95</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>38.43</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>1700</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>34.67</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>35.03</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>35.03</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>37.76</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>37.76</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>38.22</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>38.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>1800</v>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>32.42</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>38.84</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>39.32</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>1900</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>32.42</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>38.84</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>39.32</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>32.42</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>35.29</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>38.38</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>38.84</v>
+      </c>
+      <c r="I17" s="4" t="n">
+        <v>39.32</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Costo ferramenta Maico per misura (kit da regole WinPlus + voci fisse del foglio Ferramenta). Valori, non formule: rigenerare con genera_listini.py.</t>
         </is>
       </c>
     </row>

</xml_diff>